<commit_message>
switched val and test, added loss history visualization
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/tables/autoencoder_per_event_metrics.xlsx
+++ b/tables/autoencoder_per_event_metrics.xlsx
@@ -461,14 +461,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>drilling the workpiece for 15 seconds</t>
+          <t>moving towards the slot 3</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26</v>
+        <v>139</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -495,14 +495,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>drilling the workpiece for 20 seconds</t>
+          <t>dropping off the workpiece at the oven</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>82</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -529,11 +529,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>moving towards the slot 8</t>
+          <t>drilling the workpiece for 20 seconds</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -563,14 +563,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>moving towards the slot 4</t>
+          <t>milling the workpiece</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -597,11 +597,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>drilling the workpiece for 24 seconds</t>
+          <t>moving towards the slot 8</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -631,14 +631,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>moving towards the slot 3</t>
+          <t>moving towards the slot 4</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>139</v>
+        <v>65</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -665,11 +665,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lowering the workpiece</t>
+          <t>drilling the workpiece for 15 seconds</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
@@ -733,14 +733,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>milling the workpiece</t>
+          <t>lowering the workpiece</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -767,14 +767,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dropping off the workpiece at the oven</t>
+          <t>drilling the workpiece for 24 seconds</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -1413,29 +1413,29 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>burning the workpiece for 30 seconds</t>
+          <t>transporting the workpiece to the high bay warehouse</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>256</v>
+        <v>173</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1447,20 +1447,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>picking up the workpiece from the high bay warehouse waiting platform</t>
+          <t>burning the workpiece for 30 seconds</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>150</v>
+        <v>256</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1515,29 +1515,29 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>transporting the workpiece to the high bay warehouse</t>
+          <t>picking up the workpiece from the high bay warehouse waiting platform</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1821,29 +1821,29 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>transporting the bucket to the slot 8</t>
+          <t>transporting the bucket to the slot 6</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="C42" t="n">
         <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0.400</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -1855,29 +1855,29 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>transporting the bucket to the slot 6</t>
+          <t>transporting the bucket to the slot 5</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>193</v>
+        <v>101</v>
       </c>
       <c r="C43" t="n">
         <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -1957,11 +1957,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>transporting the bucket to the slot 5</t>
+          <t>transporting the bucket to the slot 8</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C46" t="n">
         <v>2</v>
@@ -2093,29 +2093,29 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ejecting the workpiece to the sink 2</t>
+          <t>dropping off the workpiece at the human workstation</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="C50" t="n">
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2161,29 +2161,29 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>dropping off the workpiece at the human workstation</t>
+          <t>ejecting the workpiece to the sink 2</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="C52" t="n">
         <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2331,29 +2331,29 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>transporting the bucket to the vacuum gripper robot crane jib</t>
+          <t>transporting the bucket to the slot 3</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="C57" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>0.286</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.375</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2399,29 +2399,29 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>transporting the bucket to the slot 3</t>
+          <t>transporting the bucket to the vacuum gripper robot crane jib</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D59" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.286</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>0.375</t>
+          <t>0.857</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2501,11 +2501,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>transporting the bucket to the high bay warehouse crane jib</t>
+          <t>ejecting the workpiece to the conveyor belt</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>159</v>
+        <v>113</v>
       </c>
       <c r="C62" t="n">
         <v>1</v>
@@ -2535,11 +2535,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ejecting the workpiece to the conveyor belt</t>
+          <t>transporting the bucket to the high bay warehouse crane jib</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>113</v>
+        <v>159</v>
       </c>
       <c r="C63" t="n">
         <v>1</v>
@@ -2671,20 +2671,20 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ejecting the workpiece to the sink 3</t>
+          <t>dropping off the workpiece at the high bay warehouse waiting platform</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2739,20 +2739,20 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>transporting the workpiece to the initial position</t>
+          <t>drilling the workpiece for 6 seconds</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>71</v>
+        <v>6</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2773,17 +2773,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>moving towards the slot 5</t>
+          <t>dropping off the workpiece at the sorting machine conveyor belt</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="C70" t="n">
         <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E70" t="n">
         <v>0</v>
@@ -2807,20 +2807,20 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>drilling the workpiece for 6 seconds</t>
+          <t>dropping off the workpiece at the drilling machine sink</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="C71" t="n">
         <v>0</v>
       </c>
       <c r="D71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2841,17 +2841,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>moving towards the punching machine sink</t>
+          <t>moving towards the slot 5</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3</v>
+        <v>71</v>
       </c>
       <c r="C72" t="n">
         <v>0</v>
       </c>
       <c r="D72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
@@ -2875,20 +2875,20 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>transporting the bucket to the slot 7</t>
+          <t>picking up the workpiece from the punching machine sink</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="C73" t="n">
         <v>0</v>
       </c>
       <c r="D73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2909,11 +2909,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>picking up the workpiece from the sink 3</t>
+          <t>moving towards the slot 6</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
@@ -3045,20 +3045,20 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>moving towards the slot 6</t>
+          <t>moving towards the slot 1</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="C78" t="n">
         <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E78" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -3079,17 +3079,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>moving towards the slot 7</t>
+          <t>picking up the workpiece from the sink 1</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="C79" t="n">
         <v>0</v>
       </c>
       <c r="D79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E79" t="n">
         <v>0</v>
@@ -3113,17 +3113,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>moving towards the slot 1</t>
+          <t>transporting the workpiece to the initial position</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>163</v>
+        <v>71</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
       </c>
       <c r="D80" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E80" t="n">
         <v>2</v>
@@ -3147,20 +3147,20 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dropping off the workpiece at the high bay warehouse waiting platform</t>
+          <t>picking up the workpiece from the sink 2</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>dropping off the workpiece at the sorting machine conveyor belt</t>
+          <t>moving towards the punching machine sink</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -3215,20 +3215,20 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>dropping off the workpiece at the drilling machine sink</t>
+          <t>moving towards the slot 7</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3249,20 +3249,20 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>picking up the workpiece from the sink 1</t>
+          <t>transporting the bucket to the slot 7</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>6</v>
+        <v>143</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3283,11 +3283,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>picking up the workpiece from the sink 2</t>
+          <t>ejecting the workpiece to the sink 3</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C85" t="n">
         <v>0</v>
@@ -3317,20 +3317,20 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>picking up the workpiece from the punching machine sink</t>
+          <t>picking up the workpiece from the sink 3</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>

</xml_diff>